<commit_message>
Fix ug Ausschalten Regel
</commit_message>
<xml_diff>
--- a/doc/COP-Berechnung.xlsx
+++ b/doc/COP-Berechnung.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
   <si>
     <t>Datum</t>
   </si>
@@ -32,23 +32,60 @@
     <t>kWh</t>
   </si>
   <si>
-    <t>MWh</t>
-  </si>
-  <si>
     <t>Wärmezähler</t>
   </si>
   <si>
     <t>Stromzähler</t>
+  </si>
+  <si>
+    <t>Diff Strom</t>
+  </si>
+  <si>
+    <t>Diff Wärme</t>
+  </si>
+  <si>
+    <t>COP</t>
+  </si>
+  <si>
+    <t>Momentanwerte</t>
+  </si>
+  <si>
+    <t>Strom</t>
+  </si>
+  <si>
+    <t>kW</t>
+  </si>
+  <si>
+    <t>Wärme</t>
+  </si>
+  <si>
+    <t>°C</t>
+  </si>
+  <si>
+    <t>Gut</t>
+  </si>
+  <si>
+    <t>Rücklauf Temp.</t>
+  </si>
+  <si>
+    <t>ca. 35</t>
+  </si>
+  <si>
+    <t>Vorlauf Temp.</t>
+  </si>
+  <si>
+    <t>Schlecht</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="dd/mm/yy;@"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="dd/mm/yy;@"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -63,8 +100,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -77,8 +122,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -95,33 +146,100 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="dotted">
+        <color auto="1"/>
+      </left>
+      <right style="dotted">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dotted">
+        <color auto="1"/>
+      </left>
+      <right style="dotted">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -402,47 +520,240 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="27.85546875" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.85546875" style="5"/>
-    <col min="2" max="2" width="27.85546875" style="9"/>
-    <col min="3" max="16384" width="27.85546875" style="6"/>
+    <col min="1" max="1" width="14.85546875" style="10" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" style="11" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" style="11" customWidth="1"/>
+    <col min="4" max="4" width="19.5703125" style="12" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" style="12" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" style="25" customWidth="1"/>
+    <col min="7" max="7" width="23.140625" style="3" customWidth="1"/>
+    <col min="8" max="16384" width="27.85546875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
+      <c r="D1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="23" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="7"/>
       <c r="B2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="5">
+      <c r="C2" s="8"/>
+      <c r="D2" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="9"/>
+      <c r="F2" s="24"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="10">
         <v>45610</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="11">
         <v>158.6</v>
       </c>
-      <c r="C3" s="6">
+      <c r="D3" s="22">
         <v>9731</v>
       </c>
+      <c r="E3" s="11"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="10">
+        <v>45613</v>
+      </c>
+      <c r="B4" s="11">
+        <v>232.65</v>
+      </c>
+      <c r="C4" s="11">
+        <f>B4-B3</f>
+        <v>74.050000000000011</v>
+      </c>
+      <c r="D4" s="22">
+        <v>9977</v>
+      </c>
+      <c r="E4" s="11">
+        <f>D4-D3</f>
+        <v>246</v>
+      </c>
+      <c r="F4" s="25">
+        <f>E4/C4</f>
+        <v>3.3220796758946651</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D5" s="22"/>
+      <c r="E5" s="11"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D6" s="22"/>
+      <c r="E6" s="11"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D7" s="22"/>
+      <c r="E7" s="11"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D8" s="22"/>
+      <c r="E8" s="11"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D9" s="22"/>
+      <c r="E9" s="11"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D10" s="22"/>
+      <c r="E10" s="11"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D11" s="22"/>
+      <c r="E11" s="11"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D12" s="22"/>
+      <c r="E12" s="11"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D13" s="22"/>
+      <c r="E13" s="11"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D14" s="22"/>
+      <c r="E14" s="11"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D15" s="22"/>
+      <c r="E15" s="11"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D16" s="22"/>
+      <c r="E16" s="11"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D17" s="22"/>
+      <c r="E17" s="11"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D18" s="22"/>
+      <c r="E18" s="11"/>
+    </row>
+    <row r="19" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="26"/>
+    </row>
+    <row r="20" spans="1:6" s="18" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="16"/>
+      <c r="B20" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" s="27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="19"/>
+      <c r="B21" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="E21" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="F21" s="28"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="11">
+        <v>2.4500000000000002</v>
+      </c>
+      <c r="E22" s="11">
+        <v>11.6</v>
+      </c>
+      <c r="F22" s="25">
+        <f>E22/D22</f>
+        <v>4.7346938775510203</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" s="11">
+        <v>3.4</v>
+      </c>
+      <c r="E24" s="11">
+        <v>9.6</v>
+      </c>
+      <c r="F24" s="25">
+        <f>E24/D24</f>
+        <v>2.8235294117647061</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D27" s="11"/>
+      <c r="E27" s="11"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.78740157480314965" bottom="0.78740157480314965" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;L&amp;Z&amp;F&amp;R&amp;D</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>